<commit_message>
Phase 2: all ten screens, 3D warehouse and TV showcase
- index.html + src/app.js (router), state.js (store adapter, replayable change batches, 6 h reset)
- Overview, PFEP table (34 columns), spreadsheet imports with cell-level report,
  PDF form ingest (pdf.js text layer, preview, inch confirmation), data fixes,
  supersession + review/apply sync, lifecycle 2x2 + planning delta,
  3D high-bay (three.js, instanced boxes, slot candidates), showcase (Red first,
  lowest DOH, loops), part lookup with source mismatches, demo guide
- lib/: pinned pdf.js 4.10.38, three.js r170 + OrbitControls, SheetJS 0.18.5 (licenses included)
- Sync no longer copies returnable container numbers: blank means one-way packaging
- High-bay placement spread across all rows
- test/e2e.py: 38 browser checks (scenarios, 390px, dark theme, console errors)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JRNkvn7B8vUCu83keAaZav
</commit_message>
<xml_diff>
--- a/samples/imports/IM-06_wh_duplicates.xlsx
+++ b/samples/imports/IM-06_wh_duplicates.xlsx
@@ -431,13 +431,13 @@
         <v>A</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E2">
         <v>1</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -451,13 +451,13 @@
         <v>A</v>
       </c>
       <c r="D3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -468,16 +468,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C4" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -488,16 +488,16 @@
         <v>High Bay</v>
       </c>
       <c r="C5" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E5">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -508,16 +508,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C6" t="str">
-        <v>A</v>
+        <v>D</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F6">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -528,16 +528,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C7" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="D7">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -548,16 +548,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C8" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F8">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -568,16 +568,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C9" t="str">
-        <v>A</v>
+        <v>F</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -588,13 +588,13 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C10" t="str">
-        <v>A</v>
+        <v>F</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F10">
         <v>1</v>
@@ -608,13 +608,13 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C11" t="str">
-        <v>A</v>
+        <v>F</v>
       </c>
       <c r="D11">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E11">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F11">
         <v>2</v>
@@ -628,16 +628,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C12" t="str">
-        <v>A</v>
+        <v>F</v>
       </c>
       <c r="D12">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
@@ -651,13 +651,13 @@
         <v>A</v>
       </c>
       <c r="D13">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
@@ -688,16 +688,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C15" t="str">
-        <v>A</v>
+        <v>E</v>
       </c>
       <c r="D15">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="E15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
@@ -708,13 +708,13 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C16" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D16">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F16">
         <v>3</v>
@@ -728,16 +728,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C17" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D17">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E17">
         <v>2</v>
       </c>
       <c r="F17">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -751,13 +751,13 @@
         <v>A</v>
       </c>
       <c r="D18">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E18">
         <v>2</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -771,13 +771,13 @@
         <v>A</v>
       </c>
       <c r="D19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -791,13 +791,13 @@
         <v>A</v>
       </c>
       <c r="D20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E20">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
@@ -814,10 +814,10 @@
         <v>4</v>
       </c>
       <c r="E21">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F21">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -828,13 +828,13 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C22" t="str">
-        <v>A</v>
+        <v>F</v>
       </c>
       <c r="D22">
+        <v>8</v>
+      </c>
+      <c r="E22">
         <v>4</v>
-      </c>
-      <c r="E22">
-        <v>2</v>
       </c>
       <c r="F22">
         <v>3</v>
@@ -848,16 +848,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C23" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
@@ -868,16 +868,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C24" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D24">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F24">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
@@ -888,16 +888,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C25" t="str">
-        <v>A</v>
+        <v>E</v>
       </c>
       <c r="D25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F25">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
@@ -908,16 +908,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C26" t="str">
-        <v>A</v>
+        <v>E</v>
       </c>
       <c r="D26">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -931,13 +931,13 @@
         <v>A</v>
       </c>
       <c r="D27">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E27">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F27">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Showcase v91: opening overview, bird's-eye return, two-leg fly-in, Pause/Prev/Next, top-5 clip export
- warehouse3d: lines A|B C|D E|F with 9 ft aisles, 24 bays x 4 lanes on level 1, pallet levels 2-5 and
  VLM towers V1-V3; moves run on a pausable clock and never pass through a rack
- showcase.js: TV showcase, single-part 'Show in 3D' from Part lookup, Export top 5 (MediaRecorder)
- tools/make-video.py renders the README clip frame by frame; docs/showcase-top5.mp4 + showcase.gif
- scrub: media files checked by embedded text, not compressed pixels
- e2e 44 checks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JRNkvn7B8vUCu83keAaZav
</commit_message>
<xml_diff>
--- a/samples/imports/IM-06_wh_duplicates.xlsx
+++ b/samples/imports/IM-06_wh_duplicates.xlsx
@@ -428,10 +428,10 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C2" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -448,10 +448,10 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C3" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -468,16 +468,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C4" t="str">
-        <v>B</v>
+        <v>E</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="E4">
         <v>1</v>
       </c>
       <c r="F4">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -488,16 +488,16 @@
         <v>High Bay</v>
       </c>
       <c r="C5" t="str">
-        <v>B</v>
+        <v>E</v>
       </c>
       <c r="D5">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="E5">
         <v>1</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -508,16 +508,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C6" t="str">
-        <v>D</v>
+        <v>B</v>
       </c>
       <c r="D6">
         <v>8</v>
       </c>
       <c r="E6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F6">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -528,16 +528,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C7" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="D7">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E7">
         <v>1</v>
       </c>
       <c r="F7">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -548,16 +548,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C8" t="str">
-        <v>C</v>
+        <v>B</v>
       </c>
       <c r="D8">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E8">
         <v>1</v>
       </c>
       <c r="F8">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9">
@@ -568,16 +568,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C9" t="str">
-        <v>F</v>
+        <v>A</v>
       </c>
       <c r="D9">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
         <v>3</v>
-      </c>
-      <c r="F9">
-        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -588,16 +588,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C10" t="str">
-        <v>F</v>
+        <v>A</v>
       </c>
       <c r="D10">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E10">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
@@ -608,16 +608,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C11" t="str">
-        <v>F</v>
+        <v>C</v>
       </c>
       <c r="D11">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F11">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
@@ -628,16 +628,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C12" t="str">
-        <v>F</v>
+        <v>A</v>
       </c>
       <c r="D12">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E12">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -651,13 +651,13 @@
         <v>A</v>
       </c>
       <c r="D13">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E13">
         <v>1</v>
       </c>
       <c r="F13">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -688,16 +688,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C15" t="str">
-        <v>E</v>
+        <v>C</v>
       </c>
       <c r="D15">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
@@ -708,16 +708,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C16" t="str">
-        <v>B</v>
+        <v>C</v>
       </c>
       <c r="D16">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F16">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -728,16 +728,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C17" t="str">
-        <v>B</v>
+        <v>D</v>
       </c>
       <c r="D17">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -748,16 +748,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C18" t="str">
-        <v>A</v>
+        <v>D</v>
       </c>
       <c r="D18">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -768,16 +768,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C19" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="D19">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F19">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
@@ -788,16 +788,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C20" t="str">
-        <v>A</v>
+        <v>C</v>
       </c>
       <c r="D20">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E20">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -808,16 +808,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C21" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="D21">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
         <v>3</v>
-      </c>
-      <c r="F21">
-        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -828,16 +828,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C22" t="str">
-        <v>F</v>
+        <v>B</v>
       </c>
       <c r="D22">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="E22">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F22">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
@@ -851,13 +851,13 @@
         <v>B</v>
       </c>
       <c r="D23">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E23">
         <v>1</v>
       </c>
       <c r="F23">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -871,13 +871,13 @@
         <v>B</v>
       </c>
       <c r="D24">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E24">
         <v>1</v>
       </c>
       <c r="F24">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
@@ -888,16 +888,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C25" t="str">
-        <v>E</v>
+        <v>B</v>
       </c>
       <c r="D25">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="E25">
         <v>1</v>
       </c>
       <c r="F25">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -908,10 +908,10 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C26" t="str">
-        <v>E</v>
+        <v>D</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -928,16 +928,16 @@
         <v>HIGHBAY</v>
       </c>
       <c r="C27" t="str">
-        <v>A</v>
+        <v>D</v>
       </c>
       <c r="D27">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="E27">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F27">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>